<commit_message>
feat(fleet): add Hook 25 and Template 04 for pre-clear session handoff protocol
</commit_message>
<xml_diff>
--- a/HOOKS_GUIDE.xlsx
+++ b/HOOKS_GUIDE.xlsx
@@ -32,6 +32,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22. خطاف قيادة وإدارة الأسطول" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23. خطاف تحويل وأتمتة سكربتات" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24. خطاف أتمتة مسارات العمل و" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25. خطاف تجميد وتسليم الجلسة " sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -473,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1471,7 +1472,49 @@
   4. **أتمتة العمليات التسويقية وتأهيل العملاء (Marketing &amp; CRM Pipelines):**
      - بناء مسارات استقبال وتحليل بيانات العملاء المحتملين من Google Ads و Facebook وتوجيه الإشعارات اللحظية عبر WhatsApp و Slack وتحديث الـ CRM.
   5. **تحصين الانقطاع ومعالجة الأخطاء (Fault Tolerance &amp; Sub-workflow Retries):**
-     - إضافة مسارات الخطأ (Error Trigger) وإعادة المحاولة مع التراجع التلقائي (Exponential Backoff) ونماذج LLM البديلة.
+     - إضافة مسارات الخطأ (Error Trigger) وإعادة المحاولة مع التراجع التلقائي (Exponential Backoff) ونماذج LLM البديلة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>25. خطاف تجميد وتسليم الجلسة قبل التصفير</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>استعد للتصفير, تجهيز clear, تجميد الجلسة, pre-clear handoff, prepare clear, freeze session, قبل التصفير</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Opus 5 (Thinking)` 
+ البديل: `Claude Sonnet 5`</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>[fleet-orchestrator], [persistent-memory-engine], [git-github-manager]</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>تجميد وتوثيق حالة الجلسة بالكامل قبل تنفيذ أمر /clear أو /compact، وتحديث ملف الحالة CURRENT_STATE.md وسجل الـ Git، وتوليد برومبت الاستئناف الفوري بنقرة واحدة لتفادي فقدان السياق عند امتلاء الجلسة (session:90%+).</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **الرصد والاستعداد للحد الحرج:** يُستدعى هذا الخطاف تلقائياً أو يدوياً عندما تبلغ الجلسة حداً مرتفعاً من الاستهلاك (مثل `session:90%` كما في طرفية Claude Code CLI أو `40%` كحد وقائي قبل تراجع جودة الذاكرة).
+  2. **تجميد وتوثيق الحالة (Freeze State):** يقوم الوكيل بمطابقة وتحديث ملف `fleet_orders/CURRENT_STATE.md` فوراً، وتوثيق آخر Commit تم اعتماده، والفرع النشط، والمهام المكتملة ونتائج بوابات الجودة (Quality Gates).
+  3. **فحص الـ Git وتأمين شجرة العمل:** التأكد من عدم وجود تعديلات عائمة أو غير محفوظة، ومزامنة أي دروس مستفادة أو ملاحظات عتادية (مثل اختناق ذاكرة R8 B-17) في `MEMORY_STORE.md`.
+  4. **تحديد خيارات المطور للمرحلة القادمة:** توضيح الخيارات والخطوة التالية المتاحة للمطور (Next Action / Next Orders) بصياغة مباشرة محددة.
+  5. **توليد برومبت الاستئناف الفوري (Resume Prompt):** طباعة برومبت جاهز للنسخ بنقرة واحدة ليلصقه المطور مباشرة في الجلسة الجديدة فور كتابة `/clear`.
+  6. **إعطاء الضوء الأخضر:** إشعار المستخدم باكتمال التجميد وإمكانية كتابة أمر `/clear` في الطرفية بأمان تام دون أي خطر لفقدان السياق.
 &lt;/div&gt;</t>
         </is>
       </c>
@@ -3170,7 +3213,109 @@
   4. **أتمتة العمليات التسويقية وتأهيل العملاء (Marketing &amp; CRM Pipelines):**
      - بناء مسارات استقبال وتحليل بيانات العملاء المحتملين من Google Ads و Facebook وتوجيه الإشعارات اللحظية عبر WhatsApp و Slack وتحديث الـ CRM.
   5. **تحصين الانقطاع ومعالجة الأخطاء (Fault Tolerance &amp; Sub-workflow Retries):**
-     - إضافة مسارات الخطأ (Error Trigger) وإعادة المحاولة مع التراجع التلقائي (Exponential Backoff) ونماذج LLM البديلة.
+     - إضافة مسارات الخطأ (Error Trigger) وإعادة المحاولة مع التراجع التلقائي (Exponential Backoff) ونماذج LLM البديلة.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>اسم الخطاف</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>المحفزات (الخطاف للنسخ)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>النموذج الأساسي والبديل</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>الوكلاء المسؤولون</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>الهدف الأساسي</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>الوصف والتفاصيل</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>25. خطاف تجميد وتسليم الجلسة قبل التصفير</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>استعد للتصفير, تجهيز clear, تجميد الجلسة, pre-clear handoff, prepare clear, freeze session, قبل التصفير</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Opus 5 (Thinking)` 
+ البديل: `Claude Sonnet 5`</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>[fleet-orchestrator], [persistent-memory-engine], [git-github-manager]</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>تجميد وتوثيق حالة الجلسة بالكامل قبل تنفيذ أمر /clear أو /compact، وتحديث ملف الحالة CURRENT_STATE.md وسجل الـ Git، وتوليد برومبت الاستئناف الفوري بنقرة واحدة لتفادي فقدان السياق عند امتلاء الجلسة (session:90%+).</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **الرصد والاستعداد للحد الحرج:** يُستدعى هذا الخطاف تلقائياً أو يدوياً عندما تبلغ الجلسة حداً مرتفعاً من الاستهلاك (مثل `session:90%` كما في طرفية Claude Code CLI أو `40%` كحد وقائي قبل تراجع جودة الذاكرة).
+  2. **تجميد وتوثيق الحالة (Freeze State):** يقوم الوكيل بمطابقة وتحديث ملف `fleet_orders/CURRENT_STATE.md` فوراً، وتوثيق آخر Commit تم اعتماده، والفرع النشط، والمهام المكتملة ونتائج بوابات الجودة (Quality Gates).
+  3. **فحص الـ Git وتأمين شجرة العمل:** التأكد من عدم وجود تعديلات عائمة أو غير محفوظة، ومزامنة أي دروس مستفادة أو ملاحظات عتادية (مثل اختناق ذاكرة R8 B-17) في `MEMORY_STORE.md`.
+  4. **تحديد خيارات المطور للمرحلة القادمة:** توضيح الخيارات والخطوة التالية المتاحة للمطور (Next Action / Next Orders) بصياغة مباشرة محددة.
+  5. **توليد برومبت الاستئناف الفوري (Resume Prompt):** طباعة برومبت جاهز للنسخ بنقرة واحدة ليلصقه المطور مباشرة في الجلسة الجديدة فور كتابة `/clear`.
+  6. **إعطاء الضوء الأخضر:** إشعار المستخدم باكتمال التجميد وإمكانية كتابة أمر `/clear` في الطرفية بأمان تام دون أي خطر لفقدان السياق.
 &lt;/div&gt;</t>
         </is>
       </c>

</xml_diff>

<commit_message>
feat(hooks): update Hook 25 to Strategic Clear and refresh prompt libraries
</commit_message>
<xml_diff>
--- a/HOOKS_GUIDE.xlsx
+++ b/HOOKS_GUIDE.xlsx
@@ -32,7 +32,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22. خطاف قيادة وإدارة الأسطول" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23. خطاف تحويل وأتمتة سكربتات" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24. خطاف أتمتة مسارات العمل و" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25. خطاف تجميد وتسليم الجلسة " sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25. خطاف التصفير الاستراتيجي " sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1482,12 +1482,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>25. خطاف تجميد وتسليم الجلسة قبل التصفير</t>
+          <t>25. خطاف التصفير الاستراتيجي وتسليم الجلسة</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>استعد للتصفير, تجهيز clear, تجميد الجلسة, pre-clear handoff, prepare clear, freeze session, قبل التصفير</t>
+          <t>التصفير الاستراتيجي, strategic clear, استعد للتصفير, تجهيز clear, تجميد الجلسة, pre-clear handoff, freeze session</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1503,18 +1503,25 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>تجميد وتوثيق حالة الجلسة بالكامل قبل تنفيذ أمر /clear أو /compact، وتحديث ملف الحالة CURRENT_STATE.md وسجل الـ Git، وتوليد برومبت الاستئناف الفوري بنقرة واحدة لتفادي فقدان السياق عند امتلاء الجلسة (session:90%+).</t>
+          <t>تقييم وإنهاء أي مهام عالقة أو ذات أولوية عاجلة لتأمين استقرار الكود، ثم تجميد وتوثيق الحالة في CURRENT_STATE.md وتوليد برومبت الاستئناف الفوري قبل تنفيذ /clear أو /compact عند امتلاء الجلسة (session:90%+).</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **الرصد والاستعداد للحد الحرج:** يُستدعى هذا الخطاف تلقائياً أو يدوياً عندما تبلغ الجلسة حداً مرتفعاً من الاستهلاك (مثل `session:90%` كما في طرفية Claude Code CLI أو `40%` كحد وقائي قبل تراجع جودة الذاكرة).
-  2. **تجميد وتوثيق الحالة (Freeze State):** يقوم الوكيل بمطابقة وتحديث ملف `fleet_orders/CURRENT_STATE.md` فوراً، وتوثيق آخر Commit تم اعتماده، والفرع النشط، والمهام المكتملة ونتائج بوابات الجودة (Quality Gates).
-  3. **فحص الـ Git وتأمين شجرة العمل:** التأكد من عدم وجود تعديلات عائمة أو غير محفوظة، ومزامنة أي دروس مستفادة أو ملاحظات عتادية (مثل اختناق ذاكرة R8 B-17) في `MEMORY_STORE.md`.
-  4. **تحديد خيارات المطور للمرحلة القادمة:** توضيح الخيارات والخطوة التالية المتاحة للمطور (Next Action / Next Orders) بصياغة مباشرة محددة.
-  5. **توليد برومبت الاستئناف الفوري (Resume Prompt):** طباعة برومبت جاهز للنسخ بنقرة واحدة ليلصقه المطور مباشرة في الجلسة الجديدة فور كتابة `/clear`.
-  6. **إعطاء الضوء الأخضر:** إشعار المستخدم باكتمال التجميد وإمكانية كتابة أمر `/clear` في الطرفية بأمان تام دون أي خطر لفقدان السياق.
+  1. **المرحلة الأولى: المسح السريع وإنهاء المهام العالقة ذات الأولوية (In-Flight Work Resolution &amp; Stabilization):**
+     - جرد فوري لأي مهام أو أوامر ذات أولوية قصوى قيد التنفيذ قبل اتخاذ قرار التصفير.
+     - إذا كانت المهمة قريبة من الإنجاز: يتم إكمالها فوراً وبناء الكود وفحصه برمجياً واعتماده بعمل `git commit` نظيف ومحكم.
+     - إذا كانت المهمة كبيرة وتحتاج جولات إضافية: يتم تثبيت الكود عند محطة استقرار آمنة (Compilable Milestone) وعزل أي تجارب ناقصة لضمان بقاء الفرع أخضر 100% وخالياً من أي أخطاء كسر بناء.
+  2. **المرحلة الثانية: تجميد الحالة وتوثيق سياق المشروع وحراسة الذاكرة (State Freeze &amp; Memory Quarantine):**
+     - مطابقة وتحديث ملف الحالة `fleet_orders/CURRENT_STATE.md` (أو `PROJECT_CONTEXT.md`) وتحديث بند "الخطوة التالية المحددة" (The One Thing To Do Next).
+     - فحص ومطابقة `git status --short --branch` للتأكد من خلو شجرة العمل من أي تعديلات تائهة أو غير معتمدة.
+     - تسجيل أي اكتشافات أو ملاحظات عتادية أو فخاخ برمجية جديدة في `MEMORY_STORE.md`.
+  3. **المرحلة الثالثة: تحديد القرارات وتوليد برومبت الاستئناف الفوري (Resume Prompt &amp; Green Light):**
+     - صياغة ملخص تسليم محكم يتضمن: ما تم إنجازه، آخر Commit معتمد، والخيارات المتاحة أمام المطور للجلسة القادمة.
+     - توليد برومبت استئناف دقيق (Ready to copy-paste) لنسخه ولصقه فور تنفيذ أمر التصفير:
+       `Read CLAUDE.md and fleet_orders/CURRENT_STATE.md. State where we are and present the choices for the next order.`
+     - منح الضوء الأخضر الصريح للمطور: تأكيد إمكانية تنفيذ أمر `/clear` أو `/compact` بأمان تام وبدون أي هدر للسياق.
 &lt;/div&gt;</t>
         </is>
       </c>
@@ -3283,12 +3290,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>25. خطاف تجميد وتسليم الجلسة قبل التصفير</t>
+          <t>25. خطاف التصفير الاستراتيجي وتسليم الجلسة</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>استعد للتصفير, تجهيز clear, تجميد الجلسة, pre-clear handoff, prepare clear, freeze session, قبل التصفير</t>
+          <t>التصفير الاستراتيجي, strategic clear, استعد للتصفير, تجهيز clear, تجميد الجلسة, pre-clear handoff, freeze session</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -3304,18 +3311,25 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تجميد وتوثيق حالة الجلسة بالكامل قبل تنفيذ أمر /clear أو /compact، وتحديث ملف الحالة CURRENT_STATE.md وسجل الـ Git، وتوليد برومبت الاستئناف الفوري بنقرة واحدة لتفادي فقدان السياق عند امتلاء الجلسة (session:90%+).</t>
+          <t>تقييم وإنهاء أي مهام عالقة أو ذات أولوية عاجلة لتأمين استقرار الكود، ثم تجميد وتوثيق الحالة في CURRENT_STATE.md وتوليد برومبت الاستئناف الفوري قبل تنفيذ /clear أو /compact عند امتلاء الجلسة (session:90%+).</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **الرصد والاستعداد للحد الحرج:** يُستدعى هذا الخطاف تلقائياً أو يدوياً عندما تبلغ الجلسة حداً مرتفعاً من الاستهلاك (مثل `session:90%` كما في طرفية Claude Code CLI أو `40%` كحد وقائي قبل تراجع جودة الذاكرة).
-  2. **تجميد وتوثيق الحالة (Freeze State):** يقوم الوكيل بمطابقة وتحديث ملف `fleet_orders/CURRENT_STATE.md` فوراً، وتوثيق آخر Commit تم اعتماده، والفرع النشط، والمهام المكتملة ونتائج بوابات الجودة (Quality Gates).
-  3. **فحص الـ Git وتأمين شجرة العمل:** التأكد من عدم وجود تعديلات عائمة أو غير محفوظة، ومزامنة أي دروس مستفادة أو ملاحظات عتادية (مثل اختناق ذاكرة R8 B-17) في `MEMORY_STORE.md`.
-  4. **تحديد خيارات المطور للمرحلة القادمة:** توضيح الخيارات والخطوة التالية المتاحة للمطور (Next Action / Next Orders) بصياغة مباشرة محددة.
-  5. **توليد برومبت الاستئناف الفوري (Resume Prompt):** طباعة برومبت جاهز للنسخ بنقرة واحدة ليلصقه المطور مباشرة في الجلسة الجديدة فور كتابة `/clear`.
-  6. **إعطاء الضوء الأخضر:** إشعار المستخدم باكتمال التجميد وإمكانية كتابة أمر `/clear` في الطرفية بأمان تام دون أي خطر لفقدان السياق.
+  1. **المرحلة الأولى: المسح السريع وإنهاء المهام العالقة ذات الأولوية (In-Flight Work Resolution &amp; Stabilization):**
+     - جرد فوري لأي مهام أو أوامر ذات أولوية قصوى قيد التنفيذ قبل اتخاذ قرار التصفير.
+     - إذا كانت المهمة قريبة من الإنجاز: يتم إكمالها فوراً وبناء الكود وفحصه برمجياً واعتماده بعمل `git commit` نظيف ومحكم.
+     - إذا كانت المهمة كبيرة وتحتاج جولات إضافية: يتم تثبيت الكود عند محطة استقرار آمنة (Compilable Milestone) وعزل أي تجارب ناقصة لضمان بقاء الفرع أخضر 100% وخالياً من أي أخطاء كسر بناء.
+  2. **المرحلة الثانية: تجميد الحالة وتوثيق سياق المشروع وحراسة الذاكرة (State Freeze &amp; Memory Quarantine):**
+     - مطابقة وتحديث ملف الحالة `fleet_orders/CURRENT_STATE.md` (أو `PROJECT_CONTEXT.md`) وتحديث بند "الخطوة التالية المحددة" (The One Thing To Do Next).
+     - فحص ومطابقة `git status --short --branch` للتأكد من خلو شجرة العمل من أي تعديلات تائهة أو غير معتمدة.
+     - تسجيل أي اكتشافات أو ملاحظات عتادية أو فخاخ برمجية جديدة في `MEMORY_STORE.md`.
+  3. **المرحلة الثالثة: تحديد القرارات وتوليد برومبت الاستئناف الفوري (Resume Prompt &amp; Green Light):**
+     - صياغة ملخص تسليم محكم يتضمن: ما تم إنجازه، آخر Commit معتمد، والخيارات المتاحة أمام المطور للجلسة القادمة.
+     - توليد برومبت استئناف دقيق (Ready to copy-paste) لنسخه ولصقه فور تنفيذ أمر التصفير:
+       `Read CLAUDE.md and fleet_orders/CURRENT_STATE.md. State where we are and present the choices for the next order.`
+     - منح الضوء الأخضر الصريح للمطور: تأكيد إمكانية تنفيذ أمر `/clear` أو `/compact` بأمان تام وبدون أي هدر للسياق.
 &lt;/div&gt;</t>
         </is>
       </c>

</xml_diff>

<commit_message>
fix(fleet): align delegation target to Antigravity CLI (agcli) and reserve Antigravity IDE for developer workbench
</commit_message>
<xml_diff>
--- a/HOOKS_GUIDE.xlsx
+++ b/HOOKS_GUIDE.xlsx
@@ -1365,11 +1365,13 @@
      - تحديد ملكية الملفات والمهام في `fleet_config.json` لمنع التصادم:
        - **Claude Code CLI** (النموذج: `Claude 5 Opus / Opus Max`): التخطيط والمراجعة المعمارية، **التنفيذ الحصري لكافة الاختبارات التلقائية**، واعتماد الأكواد وبوابات الجودة (Quality Gates).
        - **OpenCode CLI** (النموذج: `Ox Alpha Unlimited`): التنفيذ الطرفي، إدارة قواعد البيانات Drift/ORM، وعملاء الاتصال والبيانات (كتابة وبناء فقط دون تشغيل أي اختبارات).
-       - **Antigravity IDE** (النموذج: `Gemini 3.7 Flash High`): بناء الواجهات والـ Domain Logic، إدارة الذاكرة المستدامة، وهندسة السياق (كتابة وبناء فقط دون تشغيل أي اختبارات).
+       - **Antigravity CLI (`agcli`)** (النموذج: `Gemini 3.8 Flash High` / `hermes3:8b` Ollama): المنفذ الطرفي الذاتي لبناء الواجهات (UI)، تكييف المنصات، عقود الـ Domain، وهندسة الملفات (كتابة وبناء دون تشغيل اختبارات عبر سطر الأوامر دون نسخ ولصق).
+       - **Antigravity IDE** (النموذج: `Gemini 3.8 Flash High`): بيئة العمل التفاعلية وحاضنة المطور المركزية (Interactive Cockpit) لإدارة الجلسة والمحادثة واستعراض الفروقات (Diffs)؛ ولا تُوجّه أوامر تفويض الـ CLI البرمجية إليها لمنع تعليق الأتمتة.
   3. **التشغيل المباشر لأدوات الـ CLI (Headless Direct Invocation):**
      - تشغيل واستدعاء أدوات الـ CLI المثبتة مباشرة عبر سطر الأوامر غير التفاعلي:
        - استدعاء `Claude Code CLI` للمراجعة المعمارية وتشغيل الاختبارات وتدقيق الكود عبر: `claude -p "&lt;prompt&gt;"` أو `claude --print`.
        - استدعاء `OpenCode CLI` لتنفيذ الأوامر السريعة والطرفية وبناء قواعد البيانات عبر: `opencode run "&lt;message&gt;"`.
+       - استدعاء `Antigravity CLI` لمهام الواجهات وعقود الـ Domain عبر: `agcli run "&lt;message&gt;"`.
      - معالجة وإدراج مخرجات الـ CLIs تلقائياً في دورة التطوير وبوابات الجودة.
   4. **التحويل المستدام لنمط المحادثة (Session-Wide Fleet Mode Transformation):**
      - **قاعدة حاسمة:** بمجرد استدعاء وتفعيل الخطاف 22 (بالمحفزات المعتمدة أو ذكر خطاف 22)، يدخل المساعد فوراً ومستداماً في **نمط قيادة الأسطول (Fleet Command Mode)** لكامل ما تبقى من الجلسة.
@@ -2993,11 +2995,13 @@
      - تحديد ملكية الملفات والمهام في `fleet_config.json` لمنع التصادم:
        - **Claude Code CLI** (النموذج: `Claude 5 Opus / Opus Max`): التخطيط والمراجعة المعمارية، **التنفيذ الحصري لكافة الاختبارات التلقائية**، واعتماد الأكواد وبوابات الجودة (Quality Gates).
        - **OpenCode CLI** (النموذج: `Ox Alpha Unlimited`): التنفيذ الطرفي، إدارة قواعد البيانات Drift/ORM، وعملاء الاتصال والبيانات (كتابة وبناء فقط دون تشغيل أي اختبارات).
-       - **Antigravity IDE** (النموذج: `Gemini 3.7 Flash High`): بناء الواجهات والـ Domain Logic، إدارة الذاكرة المستدامة، وهندسة السياق (كتابة وبناء فقط دون تشغيل أي اختبارات).
+       - **Antigravity CLI (`agcli`)** (النموذج: `Gemini 3.8 Flash High` / `hermes3:8b` Ollama): المنفذ الطرفي الذاتي لبناء الواجهات (UI)، تكييف المنصات، عقود الـ Domain، وهندسة الملفات (كتابة وبناء دون تشغيل اختبارات عبر سطر الأوامر دون نسخ ولصق).
+       - **Antigravity IDE** (النموذج: `Gemini 3.8 Flash High`): بيئة العمل التفاعلية وحاضنة المطور المركزية (Interactive Cockpit) لإدارة الجلسة والمحادثة واستعراض الفروقات (Diffs)؛ ولا تُوجّه أوامر تفويض الـ CLI البرمجية إليها لمنع تعليق الأتمتة.
   3. **التشغيل المباشر لأدوات الـ CLI (Headless Direct Invocation):**
      - تشغيل واستدعاء أدوات الـ CLI المثبتة مباشرة عبر سطر الأوامر غير التفاعلي:
        - استدعاء `Claude Code CLI` للمراجعة المعمارية وتشغيل الاختبارات وتدقيق الكود عبر: `claude -p "&lt;prompt&gt;"` أو `claude --print`.
        - استدعاء `OpenCode CLI` لتنفيذ الأوامر السريعة والطرفية وبناء قواعد البيانات عبر: `opencode run "&lt;message&gt;"`.
+       - استدعاء `Antigravity CLI` لمهام الواجهات وعقود الـ Domain عبر: `agcli run "&lt;message&gt;"`.
      - معالجة وإدراج مخرجات الـ CLIs تلقائياً في دورة التطوير وبوابات الجودة.
   4. **التحويل المستدام لنمط المحادثة (Session-Wide Fleet Mode Transformation):**
      - **قاعدة حاسمة:** بمجرد استدعاء وتفعيل الخطاف 22 (بالمحفزات المعتمدة أو ذكر خطاف 22)، يدخل المساعد فوراً ومستداماً في **نمط قيادة الأسطول (Fleet Command Mode)** لكامل ما تبقى من الجلسة.

</xml_diff>

<commit_message>
feat(fleet): upgrade fleet baseline to Claude 5.5 (Opus Max & Sonnet 5.5), register Hook 29 & duckai-research-bridge, and enforce C-79 cross-platform path resolution
</commit_message>
<xml_diff>
--- a/HOOKS_GUIDE.xlsx
+++ b/HOOKS_GUIDE.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. خطاف خط الإنتاج البرمجي" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. خطاف التكامل الفني" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. خطاف تدقيق الصيانة" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. خطاف الفحص الأمني" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. خطاف الفحص الأمني ودرع Vi" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. خطاف مراجعة وتحديث المكتب" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. خطاف الفحص والاختبار التل" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. خطاف معالجة الأخطاء والأع" sheetId="12" state="visible" r:id="rId12"/>
@@ -36,6 +36,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26. خطاف إدارة وتحديث مكتبة ا" sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="27. خطاف الاستشارة الاستراتيج" sheetId="28" state="visible" r:id="rId28"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="28. خطاف ترحيل وتطهير أدوات ا" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="29. خطاف ترقية ومعايرة مصفوفة" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -477,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -808,12 +809,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>8. خطاف الفحص الأمني</t>
+          <t>8. خطاف الفحص الأمني ودرع Vibe Coding</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>فحص أمني, مراجعة أمان</t>
+          <t>فحص أمني, مراجعة أمان, درع الأمان, vibe security, فحص الثغرات</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -824,19 +825,26 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>[security-auditor], [code-reviewer-quality]</t>
+          <t>[security-auditor], [vibe-coding-security-shield], [code-reviewer-quality]</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>مراجعة ثغرات الأمان والتحقق من صحة المدخلات وتشفير البيانات وتأمين الوصول.</t>
+          <t>مراجعة ثغرات الأمان عبر الدرع السداسي (Semgrep, Gitleaks, Trivy, ZAP, Checkov, Renovate) وتأمين الأكواد والمفاتيح والتبعيات قبل الإنتاج.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **مصفوفة الثغرات الصارمة (VULNERABILITY MATRIX):** مسح إجباري لـ AndroidManifest والمكونات المكشوفة وتسريب البيانات.
-  2. **التحقق من صحة المدخلات وتشفير البيانات:** فحص تشفير البيانات الحساسة والجلسات وتأمين الوصول محلياً وسحابياً.</t>
+  1. **تفعيل الركائز الست لدرع الأمان (`vibe-coding-security-shield`):**
+     - **Semgrep (SAST):** فحص المنطق والأكواد المولدة بالذكاء الاصطناعي لمنع الحقن (Injection) والثغرات الإنشائية.
+     - **Gitleaks:** التحقق الصارم من انعدام تسريب المفاتيح ورموز الوصول السرية في الـ Staging وتاريخ الـ Git.
+     - **Trivy:** فحص التبعيات وصور Docker وكشف ثغرات CVEs وتوليد الـ SBOM.
+     - **OWASP ZAP (DAST):** الفحص الديناميكي للواجهات ونقاط الـ API بعد تشغيل التطبيق في بيئة الاختبار.
+     - **Checkov:** فحص أخطاء البنية التحتية والـ Misconfigurations في Dockerfile و Terraform.
+     - **Renovate:** أتمتة تحديثات التبعيات وسد الثغرات الأمنية دورياً عبر الـ PRs.
+  2. **مصفوفة الثغرات الصارمة (VULNERABILITY MATRIX):** مسح إجباري لـ AndroidManifest والمكونات المكشوفة وتسريب البيانات.
+  3. **التحقق من صحة المدخلات وتشفير البيانات:** فحص تشفير البيانات الحساسة والجلسات وتأمين الوصول محلياً وسحابياً.</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1242,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>تدقيق الجودة, فحص الكود النظيف, حراسة الجودة, clean code audit</t>
+          <t>تدقيق الجودة, فحص الكود النظيف, حراسة الجودة, clean code audit, wp guard, woo guard, debate review</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1245,18 +1253,26 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>[code-reviewer-quality], [clean-code-guard], [test-guard], [docs-guard]</t>
+          <t>[code-reviewer-quality], [clean-code-guard], [test-guard], [docs-guard], [wp-guard], [woo-guard], [debate-review]</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>تفعيل بوابات الحماية الثلاث لفحص الكود النظيف، سلامة الاختبارات، ومطابقة التوثيق.</t>
+          <t>تفعيل بوابات الحماية الشاملة للكود النظيف، سلامة الاختبارات، مطابقة التوثيق، حراسة ووردبريس وووكومرس، والمناظرة التنافسية للـ PRs.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **تفعيل بوابات الحماية الثلاث:** فحص الكود النظيف (`clean-code-guard`)، سلامة الاختبارات (`test-guard`)، ومطابقة التوثيق (`docs-guard`).</t>
+  1. **بوابات الحماية العامة للنواة (Core Guard Gates):**
+     - **الكود النظيف (`clean-code-guard`):** فحص الديف ومطابقة القواعد الـ 24 لمنع بلع الأخطاء والتعقيد الزائد والدوال الوهمية مع المراجع التخصصية.
+     - **سلامة الاختبارات (`test-guard`):** حراسة كود الاختبارات ومنع إساءة الـ Mocks وتأكيد فحص السلوك الحقيقي عبر مراجع pytest و jest و llm-app-testing.
+     - **مطابقة التوثيق (`docs-guard`):** منع الهلوسة في أسماء الدوال ومطابقة ملفات التوثيق و README مع الكود الحي.
+  2. **بوابات حراسة المنصات والتجارة الإلكترونية (Platform &amp; E-Commerce Guards):**
+     - **حراسة ووردبريس (`wp-guard`):** فحص الإضافات والقوالب، فرض التعقيم والهروب (Sanitization &amp; Escaping)، الـ Nonces، وصلاحيات المستخدم، وتأمين الاستعلامات.
+     - **حراسة ووكومرس (`woo-guard`):** حراسة العمليات المالية، منع الالتفاف على كائنات HPOS CRUD، وتأمين الـ Checkout ومطابقة معايير الدفع.
+  3. **المناظرة البرمجية التنافسية للـ Pull Requests (`debate-review`):**
+     - تشغيل مناظرة ثنائية بين نموذجين مختلفين (Main Reviewer vs Debate Reviewer) لفحص التفرعات والـ PRs وإصدار تعليقات سطرية دقيقة P0/P1/P2 خالية من النقاط العمياء.</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1287,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>استكشف المورد, حلل المستودع, تكامل المورد, scout resource, integrate repo</t>
+          <t>استكشف المورد, حلل المستودع, تكامل المورد, scout resource, integrate repo, duckai bridge, تحديث صفحة HTML, update html</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1282,18 +1298,29 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>[resource-scout-integrator], [ui-ux-pro-max], [github-talent-scout], [skill-forge-builder], [agent-optimizer], [frontend-design-builder], [git-github-manager], [powershell-runtime-pro]</t>
+          <t>[resource-scout-integrator], [duckai-research-bridge], [graft], [ui-ux-pro-max], [github-talent-scout], [skill-forge-builder], [agent-optimizer], [frontend-design-builder], [git-github-manager]</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>تحليل المستودعات الخارجية واستيراد المهارات وتعميمها وتحديث الخطافات والإكسيل وتطبيق مكتبة الأوامر ودليل hooks_user_guide.md ومزامنة المنظومة.</t>
+          <t>تحليل المستودعات الخارجية واستيراد وتعميم المهارات، وتحديث الخطافات والإكسيل والتحديث الآلي لصفحات HTML لمكتبة الأوامر التفاعلية ومزامنة المنظومة.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **استيراد وتعميم المهارات العالمية:** تحليل المستودعات الخارجية وبناء مهارات `SKILL.md` ونشرها عالمياً وتحديث المنظومة.</t>
+  1. **استيراد وتعميم المهارات العالمية:** تحليل المستودعات الخارجية وبناء مهارات `SKILL.md` ونشرها عالمياً وتحديث المنظومة.
+  2. **الحزم والموارد المعتمدة والمدمجة:**
+     - **حزمة بوابات الحراسة الشاملة (`guard-skills`):** تضم `clean-code-guard`, `test-guard`, `docs-guard`, `wp-guard`, `woo-guard` بكامل مراجعها التخصصية وموجهات OpenAI/Claude.
+     - **حزمة المراجعة التنافسية ومتابعة الـ PRs (`review-skills`):** تضم `debate-review` للمناظرة الثنائية المستقلة و `babysit-pr` للمتابعة الدورية الآلية وحل الملاحظات حتى الوصول لبوابة الدمج.
+     - **درع Vibe Coding السداسي (`vibe-coding-security-shield`):** حزم فحص Semgrep, Gitleaks, Trivy, OWASP ZAP, Checkov, Renovate لحماية الأكواد المولدة بالذكاء الاصطناعي.
+     - **مستشار هورموزي لنمو الأعمال (`hormozi-growth-advisor`):** أطر $100M Offers، معادلة القيمة، مصفوفة التوسع عبر 10 مراحل، والـ 12 Playbook.
+     - **نظام ThreeUI ثلاثي الأبعاد (`threeui-design-system`):** واجهات الويب ثلاثية الأبعاد، إضاءات الشيدر المتوهجة، ومكونات الـ 3D التفاعلية مع منع تسريب الذاكرة.
+     - **محرك سياق وخريطة الأكواد المعرفية Graft (`graft`):** بناء خرائط معرفية محلية ومستدامة عبر Tree-sitter AST لتقليل استهلاك التوكنز بنسبة 42% واستدعاءات الأدوات بنسبة 46% وتسريع استجابة Claude Code والأسطول بنسبة 60% وزيادة دقة الحلول +12 نقطة.
+     - **جسر أبحاث الذكاء الاصطناعي المجاني Duck.ai (`duckai-research-bridge`):** ربط أبحاث الويب ونماذج الاستدلال الخفيفة والمجانية (GPT-4o-mini, Claude 3 Haiku, Llama 3.3) للبحث الاستكشافي، واجهات الـ Dev/Staging لعملاء n8n و FastMCP، وحماية كوتا النماذج التجارية المدفوعة لوكالة Autovem.
+  3. **التحديث التلقائي الشامل لصفحة مكتبة الأوامر HTML (Smart Prompt Library Web View Sync):**
+     - عند استكشاف، اعتماد، أو تعديل أي خطافات جديدة في المنظومة، يُلزم الخطاف بتشغيل محرك تحديث صفحة الـ HTML (`python update_html.py`) فوراً وبشكل تلقائي.
+     - يقوم المحرك بتحليل `HOOKS_GUIDE.md` وحقن بيانات الخطافات المعتمدة (الرقم، الاسم، المحفزات، الأهداف، مستويات النماذج، الوكلاء المسؤولون، والتفاصيل الكاملة) مباشرة داخل مصفوفة `libraryData` في كافة صفحات تطبيق الويب التفاعلي لمكتبة الأوامر الذكية (`03_Dynamic_Prompt_Library/index.html`)، مع استدعاء `convert_hooks_to_sheets.py` لتحديث مصنف `HOOKS_GUIDE.xlsx`، وتوثيق الأوامر المهندسة في `مكتبة الأوامر.xlsx`.</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1388,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>[fleet-orchestrator], [code-architect], [agent-optimizer], [persistent-memory-engine]</t>
+          <t>[fleet-orchestrator], [graft], [code-architect], [agent-optimizer], [persistent-memory-engine]</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1620,7 +1647,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>[prompt-engineer], [agent-optimizer], [code-architect]</t>
+          <t>[context-governance], [graft], [prompt-engineer], [agent-optimizer], [code-architect]</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1689,7 +1716,59 @@
   3. **التدقيق التشفيري الإلزامي قبل الحذف (SHA-256 Verification):**
      - يُحظر حذف أي ملف محلي إلا بعد حساب بصمة SHA-256 للمصدر والوجهة والتأكد من التطابق التام 100%. وفي حال وجود نسخة أحدث في المركز، تُحفظ كنسخة أرشيفية.
   4. **التطهير الآمن للمشروع المحلي (Clean Workspace Guarantee):**
-     - حذف الأدوات المنقولة، وإزالة مجلد `tools/` بعد فراغه، وتنظيف مخلفات JVM (`hs_err_*.log`, `replay_*.log`) وأقفال Word المؤقتة، واستعادة الشجرة النظيفة الخالية من أي Untracked files.
+     - حذف الأدوات المنقولة، وإزالة مجلد `tools/` بعد فراغه، وتنظيف مخلفات JVM (`hs_err_*.log`, `replay_*.log`) وأقفال Word المؤقتة، واستعادة الشجرة النظيفة الخالية من أي Untracked files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>29. خطاف ترقية ومعايرة مصفوفة نماذج أسطول الـ CLIs</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>تحديث نماذج الأسطول, ترقية نماذج الأسطول, معايرة نماذج الأسطول, ترقية النماذج, تحديث مصفوفة النماذج, upgrade fleet models, calibrate fleet models, fleet model update, update fleet models</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Opus 5.5 / Opus Max (Thinking)` 
+ البديل: `Gemini 3.8 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>[fleet-orchestrator], [agent-optimizer], [code-architect], [prompt-engineer], [persistent-memory-engine]</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>ترقية ومعايرة مصفوفة نماذج أسطول الوكلاء المتعدد لاعتماد أحدث أجيال الذكاء الاصطناعي (Claude Opus 5.5 Max و Sonnet 5.5 و Gemini 3.8 Flash High و GLM 5.3 Flash و Codex GPT-5.6 Soul)، وتحديث قيود [C-11] و [C-21] و [C-38]، وتحديث ملفات fleet_config.json وقوالب التفويض، وتطبيق الويب التفاعلي ومكتبة الأوامر.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **المعايرة والترقية الشاملة لمصفوفة النماذج (Model Matrix Calibration):**
+     - ترقية نموذج القيادة المعمارية والفحص الحصري للاختبارات إلى: `Claude Opus 5.5 / Opus Max (Thinking)`.
+     - ترقية نموذج التطوير البرمجي اليومي وصناعة الميزات إلى: `Claude Sonnet 5.5`.
+     - تثبيت وتأكيد نماذج الطرفية وترشيد الكوتا: `OpenCode CLI` بنموذجي `GLM 5.3 Flash` و `Meta Muse Spark 1.3`.
+     - تثبيت منفذ واجهات Antigravity CLI / IDE: `Gemini 3.8 Flash (High Reasoning)`.
+     - تثبيت متخصص الخوارزميات والمعالجة العميقة: `Codex CLI (GPT-5.6 Soul)`.
+  2. **تحديث القيود التقنية الإلزامية (Invariants Update):**
+     - تحديث بنود [C-11] و [C-21] و [C-38] في ملف سياق الحقن الإلزامي `ACTIVE_CONTEXT_INJECTION.md`.
+  3. **المزامنة البرمجية لملفات تهيئة الأسطول (`fleet_config.json`):**
+     - فحص وتحديث حقول `active_model` في كافة ملفات `fleet_config.json` عبر المشاريع لاعتماد الجيل 5.5.
+  4. **تحديث تطبيق الويب التفاعلي والإكسيل ومكتبة الأوامر:**
+     - استدعاء `update_html.py` لتحديث مصفوفة بيانات `03_Dynamic_Prompt_Library/index.html` (29 خطافاً).
+     - استدعاء `convert_hooks_to_sheets.py` لتحديث مصنف `HOOKS_GUIDE.xlsx`.
+     - إدراج الأمر الموجه في مصنف `مكتبة الأوامر.xlsx` تحت تبويب `CLI_Core.Claude`.
+  5. **توثيق الذاكرة المستدامة (Memory Invariant):**
+     - تسجيل قرار ترقية المعمارية (ADR) في `MEMORY_STORE.md` محلياً وعالمياً.
 &lt;/div&gt;</t>
         </is>
       </c>
@@ -2847,7 +2926,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>تدقيق الجودة, فحص الكود النظيف, حراسة الجودة, clean code audit</t>
+          <t>تدقيق الجودة, فحص الكود النظيف, حراسة الجودة, clean code audit, wp guard, woo guard, debate review</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2858,18 +2937,26 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[code-reviewer-quality], [clean-code-guard], [test-guard], [docs-guard]</t>
+          <t>[code-reviewer-quality], [clean-code-guard], [test-guard], [docs-guard], [wp-guard], [woo-guard], [debate-review]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تفعيل بوابات الحماية الثلاث لفحص الكود النظيف، سلامة الاختبارات، ومطابقة التوثيق.</t>
+          <t>تفعيل بوابات الحماية الشاملة للكود النظيف، سلامة الاختبارات، مطابقة التوثيق، حراسة ووردبريس وووكومرس، والمناظرة التنافسية للـ PRs.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **تفعيل بوابات الحماية الثلاث:** فحص الكود النظيف (`clean-code-guard`)، سلامة الاختبارات (`test-guard`)، ومطابقة التوثيق (`docs-guard`).</t>
+  1. **بوابات الحماية العامة للنواة (Core Guard Gates):**
+     - **الكود النظيف (`clean-code-guard`):** فحص الديف ومطابقة القواعد الـ 24 لمنع بلع الأخطاء والتعقيد الزائد والدوال الوهمية مع المراجع التخصصية.
+     - **سلامة الاختبارات (`test-guard`):** حراسة كود الاختبارات ومنع إساءة الـ Mocks وتأكيد فحص السلوك الحقيقي عبر مراجع pytest و jest و llm-app-testing.
+     - **مطابقة التوثيق (`docs-guard`):** منع الهلوسة في أسماء الدوال ومطابقة ملفات التوثيق و README مع الكود الحي.
+  2. **بوابات حراسة المنصات والتجارة الإلكترونية (Platform &amp; E-Commerce Guards):**
+     - **حراسة ووردبريس (`wp-guard`):** فحص الإضافات والقوالب، فرض التعقيم والهروب (Sanitization &amp; Escaping)، الـ Nonces، وصلاحيات المستخدم، وتأمين الاستعلامات.
+     - **حراسة ووكومرس (`woo-guard`):** حراسة العمليات المالية، منع الالتفاف على كائنات HPOS CRUD، وتأمين الـ Checkout ومطابقة معايير الدفع.
+  3. **المناظرة البرمجية التنافسية للـ Pull Requests (`debate-review`):**
+     - تشغيل مناظرة ثنائية بين نموذجين مختلفين (Main Reviewer vs Debate Reviewer) لفحص التفرعات والـ PRs وإصدار تعليقات سطرية دقيقة P0/P1/P2 خالية من النقاط العمياء.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +3031,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>استكشف المورد, حلل المستودع, تكامل المورد, scout resource, integrate repo</t>
+          <t>استكشف المورد, حلل المستودع, تكامل المورد, scout resource, integrate repo, duckai bridge, تحديث صفحة HTML, update html</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2955,18 +3042,29 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[resource-scout-integrator], [ui-ux-pro-max], [github-talent-scout], [skill-forge-builder], [agent-optimizer], [frontend-design-builder], [git-github-manager], [powershell-runtime-pro]</t>
+          <t>[resource-scout-integrator], [duckai-research-bridge], [graft], [ui-ux-pro-max], [github-talent-scout], [skill-forge-builder], [agent-optimizer], [frontend-design-builder], [git-github-manager]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تحليل المستودعات الخارجية واستيراد المهارات وتعميمها وتحديث الخطافات والإكسيل وتطبيق مكتبة الأوامر ودليل hooks_user_guide.md ومزامنة المنظومة.</t>
+          <t>تحليل المستودعات الخارجية واستيراد وتعميم المهارات، وتحديث الخطافات والإكسيل والتحديث الآلي لصفحات HTML لمكتبة الأوامر التفاعلية ومزامنة المنظومة.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **استيراد وتعميم المهارات العالمية:** تحليل المستودعات الخارجية وبناء مهارات `SKILL.md` ونشرها عالمياً وتحديث المنظومة.</t>
+  1. **استيراد وتعميم المهارات العالمية:** تحليل المستودعات الخارجية وبناء مهارات `SKILL.md` ونشرها عالمياً وتحديث المنظومة.
+  2. **الحزم والموارد المعتمدة والمدمجة:**
+     - **حزمة بوابات الحراسة الشاملة (`guard-skills`):** تضم `clean-code-guard`, `test-guard`, `docs-guard`, `wp-guard`, `woo-guard` بكامل مراجعها التخصصية وموجهات OpenAI/Claude.
+     - **حزمة المراجعة التنافسية ومتابعة الـ PRs (`review-skills`):** تضم `debate-review` للمناظرة الثنائية المستقلة و `babysit-pr` للمتابعة الدورية الآلية وحل الملاحظات حتى الوصول لبوابة الدمج.
+     - **درع Vibe Coding السداسي (`vibe-coding-security-shield`):** حزم فحص Semgrep, Gitleaks, Trivy, OWASP ZAP, Checkov, Renovate لحماية الأكواد المولدة بالذكاء الاصطناعي.
+     - **مستشار هورموزي لنمو الأعمال (`hormozi-growth-advisor`):** أطر $100M Offers، معادلة القيمة، مصفوفة التوسع عبر 10 مراحل، والـ 12 Playbook.
+     - **نظام ThreeUI ثلاثي الأبعاد (`threeui-design-system`):** واجهات الويب ثلاثية الأبعاد، إضاءات الشيدر المتوهجة، ومكونات الـ 3D التفاعلية مع منع تسريب الذاكرة.
+     - **محرك سياق وخريطة الأكواد المعرفية Graft (`graft`):** بناء خرائط معرفية محلية ومستدامة عبر Tree-sitter AST لتقليل استهلاك التوكنز بنسبة 42% واستدعاءات الأدوات بنسبة 46% وتسريع استجابة Claude Code والأسطول بنسبة 60% وزيادة دقة الحلول +12 نقطة.
+     - **جسر أبحاث الذكاء الاصطناعي المجاني Duck.ai (`duckai-research-bridge`):** ربط أبحاث الويب ونماذج الاستدلال الخفيفة والمجانية (GPT-4o-mini, Claude 3 Haiku, Llama 3.3) للبحث الاستكشافي، واجهات الـ Dev/Staging لعملاء n8n و FastMCP، وحماية كوتا النماذج التجارية المدفوعة لوكالة Autovem.
+  3. **التحديث التلقائي الشامل لصفحة مكتبة الأوامر HTML (Smart Prompt Library Web View Sync):**
+     - عند استكشاف، اعتماد، أو تعديل أي خطافات جديدة في المنظومة، يُلزم الخطاف بتشغيل محرك تحديث صفحة الـ HTML (`python update_html.py`) فوراً وبشكل تلقائي.
+     - يقوم المحرك بتحليل `HOOKS_GUIDE.md` وحقن بيانات الخطافات المعتمدة (الرقم، الاسم، المحفزات، الأهداف، مستويات النماذج، الوكلاء المسؤولون، والتفاصيل الكاملة) مباشرة داخل مصفوفة `libraryData` في كافة صفحات تطبيق الويب التفاعلي لمكتبة الأوامر الذكية (`03_Dynamic_Prompt_Library/index.html`)، مع استدعاء `convert_hooks_to_sheets.py` لتحديث مصنف `HOOKS_GUIDE.xlsx`، وتوثيق الأوامر المهندسة في `مكتبة الأوامر.xlsx`.</t>
         </is>
       </c>
     </row>
@@ -3154,7 +3252,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[fleet-orchestrator], [code-architect], [agent-optimizer], [persistent-memory-engine]</t>
+          <t>[fleet-orchestrator], [graft], [code-architect], [agent-optimizer], [persistent-memory-engine]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -3713,7 +3811,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[prompt-engineer], [agent-optimizer], [code-architect]</t>
+          <t>[context-governance], [graft], [prompt-engineer], [agent-optimizer], [code-architect]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -3842,8 +3940,7 @@
   3. **التدقيق التشفيري الإلزامي قبل الحذف (SHA-256 Verification):**
      - يُحظر حذف أي ملف محلي إلا بعد حساب بصمة SHA-256 للمصدر والوجهة والتأكد من التطابق التام 100%. وفي حال وجود نسخة أحدث في المركز، تُحفظ كنسخة أرشيفية.
   4. **التطهير الآمن للمشروع المحلي (Clean Workspace Guarantee):**
-     - حذف الأدوات المنقولة، وإزالة مجلد `tools/` بعد فراغه، وتنظيف مخلفات JVM (`hs_err_*.log`, `replay_*.log`) وأقفال Word المؤقتة، واستعادة الشجرة النظيفة الخالية من أي Untracked files.
-&lt;/div&gt;</t>
+     - حذف الأدوات المنقولة، وإزالة مجلد `tools/` بعد فراغه، وتنظيف مخلفات JVM (`hs_err_*.log`, `replay_*.log`) وأقفال Word المؤقتة، واستعادة الشجرة النظيفة الخالية من أي Untracked files.</t>
         </is>
       </c>
     </row>
@@ -3952,6 +4049,119 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>اسم الخطاف</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>المحفزات (الخطاف للنسخ)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>النموذج الأساسي والبديل</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>الوكلاء المسؤولون</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>الهدف الأساسي</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>الوصف والتفاصيل</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>29. خطاف ترقية ومعايرة مصفوفة نماذج أسطول الـ CLIs</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>تحديث نماذج الأسطول, ترقية نماذج الأسطول, معايرة نماذج الأسطول, ترقية النماذج, تحديث مصفوفة النماذج, upgrade fleet models, calibrate fleet models, fleet model update, update fleet models</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Opus 5.5 / Opus Max (Thinking)` 
+ البديل: `Gemini 3.8 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>[fleet-orchestrator], [agent-optimizer], [code-architect], [prompt-engineer], [persistent-memory-engine]</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>ترقية ومعايرة مصفوفة نماذج أسطول الوكلاء المتعدد لاعتماد أحدث أجيال الذكاء الاصطناعي (Claude Opus 5.5 Max و Sonnet 5.5 و Gemini 3.8 Flash High و GLM 5.3 Flash و Codex GPT-5.6 Soul)، وتحديث قيود [C-11] و [C-21] و [C-38]، وتحديث ملفات fleet_config.json وقوالب التفويض، وتطبيق الويب التفاعلي ومكتبة الأوامر.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **المعايرة والترقية الشاملة لمصفوفة النماذج (Model Matrix Calibration):**
+     - ترقية نموذج القيادة المعمارية والفحص الحصري للاختبارات إلى: `Claude Opus 5.5 / Opus Max (Thinking)`.
+     - ترقية نموذج التطوير البرمجي اليومي وصناعة الميزات إلى: `Claude Sonnet 5.5`.
+     - تثبيت وتأكيد نماذج الطرفية وترشيد الكوتا: `OpenCode CLI` بنموذجي `GLM 5.3 Flash` و `Meta Muse Spark 1.3`.
+     - تثبيت منفذ واجهات Antigravity CLI / IDE: `Gemini 3.8 Flash (High Reasoning)`.
+     - تثبيت متخصص الخوارزميات والمعالجة العميقة: `Codex CLI (GPT-5.6 Soul)`.
+  2. **تحديث القيود التقنية الإلزامية (Invariants Update):**
+     - تحديث بنود [C-11] و [C-21] و [C-38] في ملف سياق الحقن الإلزامي `ACTIVE_CONTEXT_INJECTION.md`.
+  3. **المزامنة البرمجية لملفات تهيئة الأسطول (`fleet_config.json`):**
+     - فحص وتحديث حقول `active_model` في كافة ملفات `fleet_config.json` عبر المشاريع لاعتماد الجيل 5.5.
+  4. **تحديث تطبيق الويب التفاعلي والإكسيل ومكتبة الأوامر:**
+     - استدعاء `update_html.py` لتحديث مصفوفة بيانات `03_Dynamic_Prompt_Library/index.html` (29 خطافاً).
+     - استدعاء `convert_hooks_to_sheets.py` لتحديث مصنف `HOOKS_GUIDE.xlsx`.
+     - إدراج الأمر الموجه في مصنف `مكتبة الأوامر.xlsx` تحت تبويب `CLI_Core.Claude`.
+  5. **توثيق الذاكرة المستدامة (Memory Invariant):**
+     - تسجيل قرار ترقية المعمارية (ADR) في `MEMORY_STORE.md` محلياً وعالمياً.
+&lt;/div&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4510,12 +4720,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>8. خطاف الفحص الأمني</t>
+          <t>8. خطاف الفحص الأمني ودرع Vibe Coding</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>فحص أمني, مراجعة أمان</t>
+          <t>فحص أمني, مراجعة أمان, درع الأمان, vibe security, فحص الثغرات</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -4526,19 +4736,26 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[security-auditor], [code-reviewer-quality]</t>
+          <t>[security-auditor], [vibe-coding-security-shield], [code-reviewer-quality]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>مراجعة ثغرات الأمان والتحقق من صحة المدخلات وتشفير البيانات وتأمين الوصول.</t>
+          <t>مراجعة ثغرات الأمان عبر الدرع السداسي (Semgrep, Gitleaks, Trivy, ZAP, Checkov, Renovate) وتأمين الأكواد والمفاتيح والتبعيات قبل الإنتاج.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **مصفوفة الثغرات الصارمة (VULNERABILITY MATRIX):** مسح إجباري لـ AndroidManifest والمكونات المكشوفة وتسريب البيانات.
-  2. **التحقق من صحة المدخلات وتشفير البيانات:** فحص تشفير البيانات الحساسة والجلسات وتأمين الوصول محلياً وسحابياً.</t>
+  1. **تفعيل الركائز الست لدرع الأمان (`vibe-coding-security-shield`):**
+     - **Semgrep (SAST):** فحص المنطق والأكواد المولدة بالذكاء الاصطناعي لمنع الحقن (Injection) والثغرات الإنشائية.
+     - **Gitleaks:** التحقق الصارم من انعدام تسريب المفاتيح ورموز الوصول السرية في الـ Staging وتاريخ الـ Git.
+     - **Trivy:** فحص التبعيات وصور Docker وكشف ثغرات CVEs وتوليد الـ SBOM.
+     - **OWASP ZAP (DAST):** الفحص الديناميكي للواجهات ونقاط الـ API بعد تشغيل التطبيق في بيئة الاختبار.
+     - **Checkov:** فحص أخطاء البنية التحتية والـ Misconfigurations في Dockerfile و Terraform.
+     - **Renovate:** أتمتة تحديثات التبعيات وسد الثغرات الأمنية دورياً عبر الـ PRs.
+  2. **مصفوفة الثغرات الصارمة (VULNERABILITY MATRIX):** مسح إجباري لـ AndroidManifest والمكونات المكشوفة وتسريب البيانات.
+  3. **التحقق من صحة المدخلات وتشفير البيانات:** فحص تشفير البيانات الحساسة والجلسات وتأمين الوصول محلياً وسحابياً.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(hooks-library): generalize Hook 31 globally and sync 03_Dynamic_Hooks_Library app
</commit_message>
<xml_diff>
--- a/HOOKS_GUIDE.xlsx
+++ b/HOOKS_GUIDE.xlsx
@@ -37,6 +37,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="27. خطاف الاستشارة الاستراتيج" sheetId="28" state="visible" r:id="rId28"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="28. خطاف ترحيل وتطهير أدوات ا" sheetId="29" state="visible" r:id="rId29"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="29. خطاف ترقية ومعايرة مصفوفة" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30. خطاف توجيه وتفعيل الأسطول" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="31. خطاف معاينة وتنسيق العمل " sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1768,7 +1770,130 @@
      - استدعاء `convert_hooks_to_sheets.py` لتحديث مصنف `HOOKS_GUIDE.xlsx`.
      - إدراج الأمر الموجه في مصنف `مكتبة الأوامر.xlsx` تحت تبويب `CLI_Core.Claude`.
   5. **توثيق الذاكرة المستدامة (Memory Invariant):**
-     - تسجيل قرار ترقية المعمارية (ADR) في `MEMORY_STORE.md` محلياً وعالمياً.
+     - تسجيل قرار ترقية المعمارية (ADR) في `MEMORY_STORE.md` محلياً وعالمياً.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>30. خطاف توجيه وتفعيل الأسطول لأي مساحة عمل</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>وجه الأسطول, اربط الأسطول بالتطبيق, توجيه الأسطول للمشروع, استهدف هذا المشروع, target workspace fleet, fleet target app, ربط اللابتوب الثاني بالمشروع, الخطاف 30</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Opus 5.5 / Opus Max (Thinking)` 
+ البديل: `Gemini 3.8 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>[fleet-orchestrator], [devops-deployer], [code-architect], [prompt-engineer]</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>الكشف التلقائي عن مستودع مساحة العمل الحالية ونوع التقنية، وتوجيه ومزامنة عمال اللابتوب الثاني (G1, G2, G3, G4) لخدمة تطوير هذا التطبيق فورياً عبر GitHub و Tailscale مع سحب الفروع واعتمادها في قمرة القيادة.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات الآلية بمجرد إطلاق الخطاف:**
+  1. **الكشف الذكي التلقائي عن مساحة العمل الحالية (Workspace Context Discovery):**
+     - استخراج عنوان المستودع المركزي عبر `git remote get-url origin`.
+     - استخراج الفرع النشط عبر `git rev-parse --abbrev-ref HEAD` (افتراضياً `main`).
+     - اكتشاف نوع وبيئة التطبيق تلقائياً (Tech Stack): أندرويد (Compose/Kotlin)، فلاتر (Flutter)، ويب (React/Next)، أو خادم (FastAPI/Node).
+  2. **تهيئة بنية أوامر الأسطول في المشروع الحالي (Fleet Orders Scaffolding):**
+     - إنشاء مجلدات العمل التنظيمية للمشروع إن لم تكن موجودة:
+       `fleet_orders/incoming/` و `fleet_orders/in_progress/` و `fleet_orders/completed/`.
+     - إنشاء وتحديث ملف استهداف الأسطول المحلي `fleet_target.json` لتوثيق معلمات الربط للمشروع الحالي.
+  3. **بوابة الاعتماد المعماري الإلزامية لـ Claude Code قبل التوجيه (Mandatory Claude Code Pre-Dispatch Gate) [حظر صارم]:**
+     - يُحظر منعاً باتاً إرسال أو مزامنة أي توجيه أو أمر عمل إلى اللابتوب الثاني (Machine 2) إلا بعد قيام **Claude Code CLI (Opus Max)** بمراجعة وتدقيق معلمات التوجيه ومطابقة المستودع وخطة التوزيع، وإصدار وسم الاعتماد الصريح: `[APPROVED FOR REMOTE DISPATCH]`.
+     - في حال غياب الاعتماد، يظل التوجيه في حالة مسودة معلقة (`DRAFT_PENDING_CLAUDE_APPROVAL`) وتُقفل قنوات الإرسال للابتوب الثاني لحماية بيئة الإنتاج من أي استهداف خاطئ أو تسريب للملفات المحجورة.
+  4. **التوجيه والمزامنة الآلية للعقدة البعيدة (Remote Node Synchronization):**
+     - فور صدور اعتماد Claude Code، يتم فحص جاهزية اللابتوب الثاني (`python tools/remote_fleet_dispatch.py --ping`).
+     - إرسال توجيه فوري للابتوب الثاني لربط وتحديث المستودع المستهدف وسحب الفرع النشط:
+       `ssh autovem-worker-01 "cd ~/projects &amp;&amp; git remote set-url origin &lt;target_repo&gt; &amp;&amp; git fetch origin"`.
+  5. **ربط وتنشيط لوحة التحكم المركزية (Fleet Cockpit Binding :8088):**
+     - ربط خادم لوحة التحكم ([http://localhost:8088](http://localhost:8088)) بمجلد أوامر مساحة العمل الحالية.
+     - تخصيص العمال الأربعة وفقاً لطبيعة التطبيق:
+       - `Worker G1` (UI / Frontend - Jetpack Compose / Web).
+       - `Worker G2` (Backend / APIs / Domain Logic).
+       - `Worker G3` (Database / Schemas / Migrations - OpenCode Zen).
+       - `Worker G4` (Large Context / Docs / Batch).
+  6. **تأكيد سريان الضوابط المعمارية واحتكار الاختبارات [C-21]:**
+     - إلزام عمال اللابتوب الثاني بإنتاج الكود في فروع الميزات (`fleet/&lt;feature&gt;`) ودفعها لـ GitHub، مع احتكار تشغيل الاختبارات والاعتماد النهائي `[APPROVED]` لـ Claude Code CLI على جهاز المطور الرئيسي.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>31. خطاف معاينة وتنسيق العمل الجماعي لأسطول الـ CLIs</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>معاينة العمل الجماعي للأسطول, تشغيل فريق الأسطول, fleet teamwork, fleet teamwork preview, فريق عمل الأسطول, تنسيق فريق الأسطول, الخطاف 31</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Opus 5.5 / Opus Max (Thinking)` 
+ البديل: `Gemini 3.8 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>[fleet-orchestrator], [code-architect], [agent-optimizer], [test-guard], [webapp-qa-tester]</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>تفعيل وإدارة فريق عمل الأسطول الموزع (Parallel Multi-CLI Teamwork) المستوحى من هندسة teamwork-preview، لتوزيع مهام الاستكشاف، البناء، المراجعة والفحص التنافسي واحتكار الاختبارات لـ Claude Code.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>* **الفلسفة المستخلصة من الهندسة العكسية لـ Al Mustafa REA:**
+  - تحويل وتوزيع نمط العمل المتسلسل في أمر `teamwork-preview` الخاص بـ Antigravity (والذي يستهلك 7 أضعاف التوكنز داخل بيئة واحدة) إلى **فريق عمل أسطول متكامل ومتعدد الـ CLIs (Distributed Multi-CLI Teamwork)** يوزع الأدوار بذكاء واحترافية:
+    1. **قائد الأسطول والمنسق الأعلى (Master Orchestrator):** `Claude Code CLI (Opus 5.5 Max)` بالتعاون مع `Antigravity IDE` كقمرة قيادة تفاعلية وبصرية للمطور.
+    2. **مسار الاستكشاف والتفكيك المتوازي (Parallel Survey Explorers):**
+       - **المستكشف الأول (Frontend &amp; Assets):** `Antigravity CLI (agcli)` أو عامل جيميناي 1 (`Worker 1`).
+       - **المستكشف الثاني (Database &amp; Persistence):** `OpenCode CLI (GLM 5.3 Flash)` أو عامل جيميناي 2 (`Worker 2`).
+       - **المستكشف الثالث (Domain &amp; Compliance):** `OpenCode Meta Muse Spark 1.3` أو عامل جيميناي 3 (`Worker 3`).
+    3. **مسار التنفيذ الإنشائي بالدفعات (Milestone Implementation Workers):**
+       - **منفذ الواجهات:** `Antigravity CLI (agcli)` و `Cline CLI` لبناء المكونات وواجهات Compose/Web.
+       - **منفذ قواعد البيانات والخلفية:** `OpenCode CLI (GLM 5.3 Flash)` وفق قاعدة الدفعات الرباعية (Max 4 Files Per Batch) [C-78].
+       - **منفذ السقالات والسكربتات:** `OpenCode Meta Muse Spark 1.3`.
+    4. **مسار الفحص والمراجعة التنافسية (Adversarial Review &amp; Stress Testing Track):**
+       - **المراجع المعماري (Reviewer 1):** `OpenCode DeepSeek V4` لفحص الحدود المعمارية، عقود الواجهات، ومنع التكرار (DRY).
+       - **مراجع المعايير والـ RTL (Reviewer 2):** `Antigravity CLI (agcli)` لفحص التوافق اللغوي وتنسيق BiDi/RTL وسلامة معرفات DOM.
+       - **المتحدي الأول (Challenger 1):** `OpenCode CLI` لتوليد واختبار سيناريوهات الضغط والحدود القصوى للبيانات.
+       - **المتحدي الثاني (Challenger 2 - Browser QA):** `Antigravity CLI (agcli)` مع مهارة `webapp-qa-tester` (Playwright / Chrome DevTools) لفحص المتصفح الحقيقي بتكلفة $0.00 وفق القيد [C-96].
+    5. **المحقق الجنائي والاحتكار الحصري للاختبارات (Forensic Auditor &amp; Exclusive Test Monopoly):**
+       - `Claude Code CLI (Opus Max)` ينفذ الاختبارات التلقائية حصرياً (`unit`, `integration`, `e2e`) ويتحقق من انعدام التزييف (Zero Facades / Genuine Byte Sizes) ويصدر ختم الاعتماد الرسمي `[APPROVED]` في `GATE_STATUS.md`.
+* **طريقة العمل والإجراءات الآلية (Execution Flow):**
+  1. **التهيئة وسقالة مساحة العمل (`init`):**
+     - تشغيل `python tools/fleet_teamwork_orchestrator.py init --name "&lt;Project&gt;" --objective "&lt;Goal&gt;"`.
+     - إنشاء مجلد `.agents/fleet_teamwork/` وضمان اقتصاره الصارم على البيانات الوصفية (Metadata-Only) دون أي ملفات كود أو نسخ ثنائية.
+  2. **توليد أوامر التفويض المعيارية (`delegate`):**
+     - توليد موجهات التفويض للمنفذين باللغة الإنجليزية طبقاً لـ `Template 02: Task Delegation Protocol`.
+     - ضخ الموجهات عبر قنوات التدفق `stdin` بترميز UTF-8 طبقاً للقيد [C-91].
+  3. **إدارة البوابات وتوثيق القرارات (`verdict` &amp; `status`):**
+     - تحديث حالات البوابات في `GATE_STATUS.md` بعد كل جولة فحص (PASS / FAIL / FIX_REQUIRED).
+     - توثيق الدروس المستفادة والقرارات المعمارية في `MEMORY_STORE.md` محلياً وعالمياً.
 &lt;/div&gt;</t>
         </is>
       </c>
@@ -4152,7 +4277,250 @@
      - استدعاء `convert_hooks_to_sheets.py` لتحديث مصنف `HOOKS_GUIDE.xlsx`.
      - إدراج الأمر الموجه في مصنف `مكتبة الأوامر.xlsx` تحت تبويب `CLI_Core.Claude`.
   5. **توثيق الذاكرة المستدامة (Memory Invariant):**
-     - تسجيل قرار ترقية المعمارية (ADR) في `MEMORY_STORE.md` محلياً وعالمياً.
+     - تسجيل قرار ترقية المعمارية (ADR) في `MEMORY_STORE.md` محلياً وعالمياً.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>اسم الخطاف</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>المحفزات (الخطاف للنسخ)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>النموذج الأساسي والبديل</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>الوكلاء المسؤولون</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>الهدف الأساسي</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>الوصف والتفاصيل</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>30. خطاف توجيه وتفعيل الأسطول لأي مساحة عمل</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>وجه الأسطول, اربط الأسطول بالتطبيق, توجيه الأسطول للمشروع, استهدف هذا المشروع, target workspace fleet, fleet target app, ربط اللابتوب الثاني بالمشروع, الخطاف 30</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Opus 5.5 / Opus Max (Thinking)` 
+ البديل: `Gemini 3.8 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>[fleet-orchestrator], [devops-deployer], [code-architect], [prompt-engineer]</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>الكشف التلقائي عن مستودع مساحة العمل الحالية ونوع التقنية، وتوجيه ومزامنة عمال اللابتوب الثاني (G1, G2, G3, G4) لخدمة تطوير هذا التطبيق فورياً عبر GitHub و Tailscale مع سحب الفروع واعتمادها في قمرة القيادة.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات الآلية بمجرد إطلاق الخطاف:**
+  1. **الكشف الذكي التلقائي عن مساحة العمل الحالية (Workspace Context Discovery):**
+     - استخراج عنوان المستودع المركزي عبر `git remote get-url origin`.
+     - استخراج الفرع النشط عبر `git rev-parse --abbrev-ref HEAD` (افتراضياً `main`).
+     - اكتشاف نوع وبيئة التطبيق تلقائياً (Tech Stack): أندرويد (Compose/Kotlin)، فلاتر (Flutter)، ويب (React/Next)، أو خادم (FastAPI/Node).
+  2. **تهيئة بنية أوامر الأسطول في المشروع الحالي (Fleet Orders Scaffolding):**
+     - إنشاء مجلدات العمل التنظيمية للمشروع إن لم تكن موجودة:
+       `fleet_orders/incoming/` و `fleet_orders/in_progress/` و `fleet_orders/completed/`.
+     - إنشاء وتحديث ملف استهداف الأسطول المحلي `fleet_target.json` لتوثيق معلمات الربط للمشروع الحالي.
+  3. **بوابة الاعتماد المعماري الإلزامية لـ Claude Code قبل التوجيه (Mandatory Claude Code Pre-Dispatch Gate) [حظر صارم]:**
+     - يُحظر منعاً باتاً إرسال أو مزامنة أي توجيه أو أمر عمل إلى اللابتوب الثاني (Machine 2) إلا بعد قيام **Claude Code CLI (Opus Max)** بمراجعة وتدقيق معلمات التوجيه ومطابقة المستودع وخطة التوزيع، وإصدار وسم الاعتماد الصريح: `[APPROVED FOR REMOTE DISPATCH]`.
+     - في حال غياب الاعتماد، يظل التوجيه في حالة مسودة معلقة (`DRAFT_PENDING_CLAUDE_APPROVAL`) وتُقفل قنوات الإرسال للابتوب الثاني لحماية بيئة الإنتاج من أي استهداف خاطئ أو تسريب للملفات المحجورة.
+  4. **التوجيه والمزامنة الآلية للعقدة البعيدة (Remote Node Synchronization):**
+     - فور صدور اعتماد Claude Code، يتم فحص جاهزية اللابتوب الثاني (`python tools/remote_fleet_dispatch.py --ping`).
+     - إرسال توجيه فوري للابتوب الثاني لربط وتحديث المستودع المستهدف وسحب الفرع النشط:
+       `ssh autovem-worker-01 "cd ~/projects &amp;&amp; git remote set-url origin &lt;target_repo&gt; &amp;&amp; git fetch origin"`.
+  5. **ربط وتنشيط لوحة التحكم المركزية (Fleet Cockpit Binding :8088):**
+     - ربط خادم لوحة التحكم ([http://localhost:8088](http://localhost:8088)) بمجلد أوامر مساحة العمل الحالية.
+     - تخصيص العمال الأربعة وفقاً لطبيعة التطبيق:
+       - `Worker G1` (UI / Frontend - Jetpack Compose / Web).
+       - `Worker G2` (Backend / APIs / Domain Logic).
+       - `Worker G3` (Database / Schemas / Migrations - OpenCode Zen).
+       - `Worker G4` (Large Context / Docs / Batch).
+  6. **تأكيد سريان الضوابط المعمارية واحتكار الاختبارات [C-21]:**
+     - إلزام عمال اللابتوب الثاني بإنتاج الكود في فروع الميزات (`fleet/&lt;feature&gt;`) ودفعها لـ GitHub، مع احتكار تشغيل الاختبارات والاعتماد النهائي `[APPROVED]` لـ Claude Code CLI على جهاز المطور الرئيسي.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>اسم الخطاف</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>المحفزات (الخطاف للنسخ)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>النموذج الأساسي والبديل</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>الوكلاء المسؤولون</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>الهدف الأساسي</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>الوصف والتفاصيل</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>31. خطاف معاينة وتنسيق العمل الجماعي لأسطول الـ CLIs</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>معاينة العمل الجماعي للأسطول, تشغيل فريق الأسطول, fleet teamwork, fleet teamwork preview, فريق عمل الأسطول, تنسيق فريق الأسطول, الخطاف 31</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Opus 5.5 / Opus Max (Thinking)` 
+ البديل: `Gemini 3.8 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>[fleet-orchestrator], [code-architect], [agent-optimizer], [test-guard], [webapp-qa-tester]</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>تفعيل وإدارة فريق عمل الأسطول الموزع (Parallel Multi-CLI Teamwork) المستوحى من هندسة teamwork-preview، لتوزيع مهام الاستكشاف، البناء، المراجعة والفحص التنافسي واحتكار الاختبارات لـ Claude Code.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>* **الفلسفة المستخلصة من الهندسة العكسية لـ Al Mustafa REA:**
+  - تحويل وتوزيع نمط العمل المتسلسل في أمر `teamwork-preview` الخاص بـ Antigravity (والذي يستهلك 7 أضعاف التوكنز داخل بيئة واحدة) إلى **فريق عمل أسطول متكامل ومتعدد الـ CLIs (Distributed Multi-CLI Teamwork)** يوزع الأدوار بذكاء واحترافية:
+    1. **قائد الأسطول والمنسق الأعلى (Master Orchestrator):** `Claude Code CLI (Opus 5.5 Max)` بالتعاون مع `Antigravity IDE` كقمرة قيادة تفاعلية وبصرية للمطور.
+    2. **مسار الاستكشاف والتفكيك المتوازي (Parallel Survey Explorers):**
+       - **المستكشف الأول (Frontend &amp; Assets):** `Antigravity CLI (agcli)` أو عامل جيميناي 1 (`Worker 1`).
+       - **المستكشف الثاني (Database &amp; Persistence):** `OpenCode CLI (GLM 5.3 Flash)` أو عامل جيميناي 2 (`Worker 2`).
+       - **المستكشف الثالث (Domain &amp; Compliance):** `OpenCode Meta Muse Spark 1.3` أو عامل جيميناي 3 (`Worker 3`).
+    3. **مسار التنفيذ الإنشائي بالدفعات (Milestone Implementation Workers):**
+       - **منفذ الواجهات:** `Antigravity CLI (agcli)` و `Cline CLI` لبناء المكونات وواجهات Compose/Web.
+       - **منفذ قواعد البيانات والخلفية:** `OpenCode CLI (GLM 5.3 Flash)` وفق قاعدة الدفعات الرباعية (Max 4 Files Per Batch) [C-78].
+       - **منفذ السقالات والسكربتات:** `OpenCode Meta Muse Spark 1.3`.
+    4. **مسار الفحص والمراجعة التنافسية (Adversarial Review &amp; Stress Testing Track):**
+       - **المراجع المعماري (Reviewer 1):** `OpenCode DeepSeek V4` لفحص الحدود المعمارية، عقود الواجهات، ومنع التكرار (DRY).
+       - **مراجع المعايير والـ RTL (Reviewer 2):** `Antigravity CLI (agcli)` لفحص التوافق اللغوي وتنسيق BiDi/RTL وسلامة معرفات DOM.
+       - **المتحدي الأول (Challenger 1):** `OpenCode CLI` لتوليد واختبار سيناريوهات الضغط والحدود القصوى للبيانات.
+       - **المتحدي الثاني (Challenger 2 - Browser QA):** `Antigravity CLI (agcli)` مع مهارة `webapp-qa-tester` (Playwright / Chrome DevTools) لفحص المتصفح الحقيقي بتكلفة $0.00 وفق القيد [C-96].
+    5. **المحقق الجنائي والاحتكار الحصري للاختبارات (Forensic Auditor &amp; Exclusive Test Monopoly):**
+       - `Claude Code CLI (Opus Max)` ينفذ الاختبارات التلقائية حصرياً (`unit`, `integration`, `e2e`) ويتحقق من انعدام التزييف (Zero Facades / Genuine Byte Sizes) ويصدر ختم الاعتماد الرسمي `[APPROVED]` في `GATE_STATUS.md`.
+* **طريقة العمل والإجراءات الآلية (Execution Flow):**
+  1. **التهيئة وسقالة مساحة العمل (`init`):**
+     - تشغيل `python tools/fleet_teamwork_orchestrator.py init --name "&lt;Project&gt;" --objective "&lt;Goal&gt;"`.
+     - إنشاء مجلد `.agents/fleet_teamwork/` وضمان اقتصاره الصارم على البيانات الوصفية (Metadata-Only) دون أي ملفات كود أو نسخ ثنائية.
+  2. **توليد أوامر التفويض المعيارية (`delegate`):**
+     - توليد موجهات التفويض للمنفذين باللغة الإنجليزية طبقاً لـ `Template 02: Task Delegation Protocol`.
+     - ضخ الموجهات عبر قنوات التدفق `stdin` بترميز UTF-8 طبقاً للقيد [C-91].
+  3. **إدارة البوابات وتوثيق القرارات (`verdict` &amp; `status`):**
+     - تحديث حالات البوابات في `GATE_STATUS.md` بعد كل جولة فحص (PASS / FAIL / FIX_REQUIRED).
+     - توثيق الدروس المستفادة والقرارات المعمارية في `MEMORY_STORE.md` محلياً وعالمياً.
 &lt;/div&gt;</t>
         </is>
       </c>

</xml_diff>